<commit_message>
Revise reviewer release files
</commit_message>
<xml_diff>
--- a/results/final_sdss32_provenance/final_sdss32_provenance.xlsx
+++ b/results/final_sdss32_provenance/final_sdss32_provenance.xlsx
@@ -536,7 +536,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>SDSS3.2-Final</t>
+          <t>SDSS</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -597,7 +597,7 @@
       </c>
       <c r="S2" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dn_sdss32_final_profile_summary_20260519_002234.csv</t>
+          <t>results/archived_profile_grid/dn_sdss32_final_profile_summary_20260519_002234.csv</t>
         </is>
       </c>
     </row>
@@ -609,7 +609,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>SDSS3.2-Final</t>
+          <t>SDSS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -670,7 +670,7 @@
       </c>
       <c r="S3" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/df_sdss32_final_profile_summary_20260519_041636.csv</t>
+          <t>results/archived_profile_grid/df_sdss32_final_profile_summary_20260519_041636.csv</t>
         </is>
       </c>
     </row>
@@ -682,7 +682,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>SDSS3.2-Final</t>
+          <t>SDSS</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -743,7 +743,7 @@
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dpn_sdss32_final_profile_summary_20260519_121738.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_summary_20260519_121738.csv</t>
         </is>
       </c>
     </row>
@@ -755,7 +755,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SDSS3.2-Final</t>
+          <t>SDSS</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="S5" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dka_sdss32_final_profile_summary_20260519_131725.csv</t>
+          <t>results/archived_profile_grid/dka_sdss32_final_profile_summary_20260519_131725.csv</t>
         </is>
       </c>
     </row>
@@ -842,7 +842,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>SDSS3.2-Final</t>
+          <t>SDSS</t>
         </is>
       </c>
     </row>
@@ -916,7 +916,7 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>SDSS3.2-Final</t>
+          <t>SDSS</t>
         </is>
       </c>
     </row>
@@ -1137,7 +1137,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dn_sdss32_final_profile_detail_20260519_002234.csv</t>
+          <t>results/archived_profile_grid/dn_sdss32_final_profile_detail_20260519_002234.csv</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1238,7 +1238,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dn_sdss32_final_profile_detail_20260519_002234.csv</t>
+          <t>results/archived_profile_grid/dn_sdss32_final_profile_detail_20260519_002234.csv</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1339,7 +1339,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dn_sdss32_final_profile_detail_20260519_002234.csv</t>
+          <t>results/archived_profile_grid/dn_sdss32_final_profile_detail_20260519_002234.csv</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1440,7 +1440,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dn_sdss32_final_profile_detail_20260519_002234.csv</t>
+          <t>results/archived_profile_grid/dn_sdss32_final_profile_detail_20260519_002234.csv</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1541,7 +1541,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dn_sdss32_final_profile_detail_20260519_002234.csv</t>
+          <t>results/archived_profile_grid/dn_sdss32_final_profile_detail_20260519_002234.csv</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1743,7 +1743,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1945,7 +1945,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2147,7 +2147,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dka_sdss32_final_profile_detail_20260519_131725.csv</t>
+          <t>results/archived_profile_grid/dka_sdss32_final_profile_detail_20260519_131725.csv</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -2248,7 +2248,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dka_sdss32_final_profile_detail_20260519_131725.csv</t>
+          <t>results/archived_profile_grid/dka_sdss32_final_profile_detail_20260519_131725.csv</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -2349,7 +2349,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dka_sdss32_final_profile_detail_20260519_131725.csv</t>
+          <t>results/archived_profile_grid/dka_sdss32_final_profile_detail_20260519_131725.csv</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -2450,7 +2450,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dka_sdss32_final_profile_detail_20260519_131725.csv</t>
+          <t>results/archived_profile_grid/dka_sdss32_final_profile_detail_20260519_131725.csv</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -2551,7 +2551,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>/mnt/data/sdss_github_release/results/archived_profile_grid/dka_sdss32_final_profile_detail_20260519_131725.csv</t>
+          <t>results/archived_profile_grid/dka_sdss32_final_profile_detail_20260519_131725.csv</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">

</xml_diff>

<commit_message>
Revise reproducibility documentation and model code
</commit_message>
<xml_diff>
--- a/results/final_sdss32_provenance/final_sdss32_provenance.xlsx
+++ b/results/final_sdss32_provenance/final_sdss32_provenance.xlsx
@@ -1642,7 +1642,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_121738.csv</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1731,7 +1731,7 @@
       </c>
       <c r="AC7" t="inlineStr">
         <is>
-          <t>outputs\dpn_sdss32_final_s8_h0p60_m0p20_e0p20_seed42_20260519_065539\20260519_084752</t>
+          <t>outputs\dpn_sdss32_final_s8_h0p60_m0p20_e0p20_seed42_20260519_121738\20260519_144239</t>
         </is>
       </c>
     </row>
@@ -1743,7 +1743,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_121738.csv</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1832,7 +1832,7 @@
       </c>
       <c r="AC8" t="inlineStr">
         <is>
-          <t>outputs\dpn_sdss32_final_s8_h0p60_m0p20_e0p20_seed52_20260519_065539\20260519_084831</t>
+          <t>outputs\dpn_sdss32_final_s8_h0p60_m0p20_e0p20_seed52_20260519_121738\20260519_144335</t>
         </is>
       </c>
     </row>
@@ -1844,7 +1844,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_121738.csv</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1933,7 +1933,7 @@
       </c>
       <c r="AC9" t="inlineStr">
         <is>
-          <t>outputs\dpn_sdss32_final_s8_h0p60_m0p20_e0p20_seed62_20260519_065539\20260519_084911</t>
+          <t>outputs\dpn_sdss32_final_s8_h0p60_m0p20_e0p20_seed62_20260519_121738\20260519_144418</t>
         </is>
       </c>
     </row>
@@ -1945,7 +1945,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_121738.csv</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -2034,7 +2034,7 @@
       </c>
       <c r="AC10" t="inlineStr">
         <is>
-          <t>outputs\dpn_sdss32_final_s8_h0p60_m0p20_e0p20_seed72_20260519_065539\20260519_084948</t>
+          <t>outputs\dpn_sdss32_final_s8_h0p60_m0p20_e0p20_seed72_20260519_121738\20260519_144501</t>
         </is>
       </c>
     </row>
@@ -2046,7 +2046,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_065539.csv</t>
+          <t>results/archived_profile_grid/dpn_sdss32_final_profile_detail_20260519_121738.csv</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -2135,7 +2135,7 @@
       </c>
       <c r="AC11" t="inlineStr">
         <is>
-          <t>outputs\dpn_sdss32_final_s8_h0p60_m0p20_e0p20_seed82_20260519_065539\20260519_085025</t>
+          <t>outputs\dpn_sdss32_final_s8_h0p60_m0p20_e0p20_seed82_20260519_121738\20260519_144543</t>
         </is>
       </c>
     </row>

</xml_diff>